<commit_message>
feat(home): timeline item4 改寫 + FAQ Q7 改回簡短版
- 重要時程 item4「禪修正式開始 / 報到、安單...」→「報到、入住後 / 展開為期五日四夜的四念處禪修」
- FAQ Q7「費用大約多少？」→「禪修需要費用嗎？」答覆改為簡短兩行版

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/客戶交付/表單文案.xlsx
+++ b/docs/客戶交付/表單文案.xlsx
@@ -467,13 +467,13 @@
     <t>home.timeline.item4.title</t>
   </si>
   <si>
-    <t>禪修正式開始</t>
+    <t>報到、入住後</t>
   </si>
   <si>
     <t>home.timeline.item4.desc</t>
   </si>
   <si>
-    <t>報到、安單、開始為期五日四夜的四念處禪修。</t>
+    <t>展開為期五日四夜的四念處禪修</t>
   </si>
   <si>
     <t>首頁 &gt; FAQ</t>
@@ -632,13 +632,13 @@
     <t>home.faq.q7.title</t>
   </si>
   <si>
-    <t>費用大約多少？</t>
+    <t>禪修需要費用嗎？</t>
   </si>
   <si>
     <t>home.faq.q7.answer</t>
   </si>
   <si>
-    <t>禪修課程本身免費。食宿、場地及交通等費用依房型由參加者自理，具體金額會在錄取通知中載明，並由學員專區完成登記繳費。</t>
+    <t>禪修課程免費。學員需負擔食宿等相關費用</t>
   </si>
   <si>
     <t>首頁 &gt; FAQ &gt; Q8</t>
@@ -11436,7 +11436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="12" t="s">
         <v>199</v>
       </c>

</xml_diff>